<commit_message>
Playwright automation assignment completed
</commit_message>
<xml_diff>
--- a/playwright_whatsapp_bot/contacts.xlsx
+++ b/playwright_whatsapp_bot/contacts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Projects\Gen AI Program\playwright_whatsapp_bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16659122-9800-4435-8B70-FC79AB5F26C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D19702E0-E7AC-4166-999F-1E9A2019DEF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{4030D962-6643-40B0-9EA0-EF2FD3336B5D}"/>
   </bookViews>
@@ -39,9 +39,6 @@
     <t>My.no.prvs</t>
   </si>
   <si>
-    <t>Test</t>
-  </si>
-  <si>
     <t>Name</t>
   </si>
   <si>
@@ -49,6 +46,9 @@
   </si>
   <si>
     <t>Message</t>
+  </si>
+  <si>
+    <t>How was your day?</t>
   </si>
 </sst>
 </file>
@@ -409,13 +409,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>3</v>
-      </c>
-      <c r="C1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -426,7 +426,7 @@
         <v>9884917471</v>
       </c>
       <c r="C2" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>